<commit_message>
Add footprints for remaining parts
</commit_message>
<xml_diff>
--- a/hardware/hardware_bom.xlsx
+++ b/hardware/hardware_bom.xlsx
@@ -11,6 +11,9 @@
     <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="ILIM_Calculator" sheetId="2" state="visible" r:id="rId4"/>
   </sheets>
+  <definedNames>
+    <definedName function="false" hidden="true" localSheetId="0" name="_xlnm._FilterDatabase" vbProcedure="false">Sheet1!$A$10:$G$56</definedName>
+  </definedNames>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.001"/>
   <extLst>
     <ext xmlns:loext="http://schemas.libreoffice.org/" uri="{7626C862-2A13-11E5-B345-FEFF819CDC9F}">
@@ -21,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="101" uniqueCount="95">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="195">
   <si>
     <t xml:space="preserve">Part Number</t>
   </si>
@@ -56,15 +59,27 @@
     <t xml:space="preserve">https://www.digikey.com/short/59jf1dn5</t>
   </si>
   <si>
-    <t xml:space="preserve">RA1113112R</t>
-  </si>
-  <si>
-    <t xml:space="preserve">switch rocker</t>
+    <t xml:space="preserve">D6R90 F2 LFS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Push-button</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/hdhnn44w</t>
   </si>
   <si>
     <t xml:space="preserve">https://www.digikey.com/short/79brjhhr</t>
   </si>
   <si>
+    <t xml:space="preserve">PTS636SK25FSMTR LFS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">tactile switch</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/tqpwv0vc</t>
+  </si>
+  <si>
     <t xml:space="preserve">ESP32-S3-WROOM-1-N8R8</t>
   </si>
   <si>
@@ -98,6 +113,15 @@
     <t xml:space="preserve">https://www.digikey.com/short/pm4rdwd2</t>
   </si>
   <si>
+    <t xml:space="preserve">UJ20-C-H-G-SMT-1-P16-TR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Usb-c 2.0 16pin</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/8wf2qdw7</t>
+  </si>
+  <si>
     <t xml:space="preserve">TSD05DYFR</t>
   </si>
   <si>
@@ -158,6 +182,276 @@
     <t xml:space="preserve">https://www.digikey.com/short/9wmrww28</t>
   </si>
   <si>
+    <t xml:space="preserve">TPS63802DLAR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3.3V 2A buck-boost regulator</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/rn7hwcbv</t>
+  </si>
+  <si>
+    <t xml:space="preserve">regulator inductor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">IHLP2020CZERR47M11</t>
+  </si>
+  <si>
+    <t xml:space="preserve">.47uH, 6ohm DCR, shielded, 9A saturation, 14A current rating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/dr2t2rh3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">VLS5045EX-1R0N</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1uH, 19.5ohm, shielded, 8.9A saturation, </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/bzn0tcvb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM21BZ71A226ME15L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">22uF +-20%, 10V, X7R 0805 cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/mf2tfnjj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM21BR71A106KA73L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10uF +-10%, 10V, X7R 0805 cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/rt57p4qm</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM21BR71C105KA01L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 uF +=10%, 16V, X7R, 0805 cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/7hz15vf8</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CC0805KRX7R9BB104</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.1uF +-10%, 50V, X7R 0805 cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/rr75tjc7</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CL21B473KBCNNNC</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47nF +-10%, 50V, X7R 0805 cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/4h9c3bdn</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GRM21BR71C475KE51L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.7UF +-10%, 16V, X7R 0805 cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/530vpb41</t>
+  </si>
+  <si>
+    <t xml:space="preserve">LTST-C171KGKT</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2vf, 0805 green smd led</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/fj545nf5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-0710ML</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10Mohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/bbhz3zv5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-07909KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">909kohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/9htt0t5p</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-07511KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">511kohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/htrpqnwb</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-07200KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200kohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/87t4pmvj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-07100KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">100kohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/8zrcqwv1</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-0791KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">291kohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/jz0j7qwj</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-0747KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">47kohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/t783tv8q</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-072KL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2kohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/j372f423</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-074K7L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">4.7ohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/qqztb447</t>
+  </si>
+  <si>
+    <t xml:space="preserve">CRCW08055K36FKEA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5.36kohm, +-1%, 1/4W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/fwtnq4t2</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-0731K6L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">31.6kohm, +-1%, 1/4W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/q7r44q7j</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RMCF0805FT10K0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10kohm, +-1%, 1/8W, 0805 resistor</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/8p9d02w5</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RT0805BRD078K25L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">8.25kohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/7pr3bpp9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-071K05L</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1.05kohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/m193bvhf</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-07499RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">499ohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/84d3dtz0</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805JR-07330RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">330ohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/2q2wzv75</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-07432RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">432ohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/d7dnf71h</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805FR-07200RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">200ohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/hqnnnh0b</t>
+  </si>
+  <si>
+    <t xml:space="preserve">RC0805JR-070RL</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0ohm, +-1%, 1/8W, 0805 smd</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/m502crn9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 pos, wire to board, phoenix contact, horizontal</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/fn8z8mcd</t>
+  </si>
+  <si>
     <t xml:space="preserve">Backup Parts</t>
   </si>
   <si>
@@ -189,6 +483,15 @@
   </si>
   <si>
     <t xml:space="preserve">https://www.digikey.com/short/fd05pjh9</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BCL3520FT-R47M-D</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.47uH inductor, 8A saturation, 6mOhm DCR</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.digikey.com/short/w5fbzjmj</t>
   </si>
   <si>
     <t xml:space="preserve">USB-C ILIM Calculator</t>
@@ -510,7 +813,7 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="true" indent="0" shrinkToFit="false"/>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="164" fontId="5" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
@@ -607,7 +910,22 @@
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
     <cellStyle name="Normal" xfId="20"/>
   </cellStyles>
-  <dxfs count="2">
+  <dxfs count="4">
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFDDDDDD"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
     <dxf>
       <font>
         <name val="Arial"/>
@@ -694,6 +1012,10 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -807,7 +1129,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="B10:J45"/>
+  <dimension ref="A10:J75"/>
   <sheetFormatPr defaultColWidth="11.53515625" defaultRowHeight="12.8" customHeight="true" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="1" width="27.48"/>
@@ -869,419 +1191,1082 @@
         <v>12</v>
       </c>
       <c r="D12" s="1" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="E12" s="1" t="n">
-        <v>0.64</v>
+        <v>1.56</v>
       </c>
       <c r="F12" s="3" t="n">
         <f aca="false">D12*E12</f>
-        <v>0.64</v>
+        <v>4.68</v>
       </c>
       <c r="G12" s="1" t="s">
         <v>13</v>
       </c>
-    </row>
-    <row r="13" customFormat="false" ht="23.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="J12" s="1" t="s">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B13" s="1" t="s">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="C13" s="4" t="s">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="D13" s="1" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E13" s="1" t="n">
-        <v>6.13</v>
+        <v>0.25</v>
       </c>
       <c r="F13" s="3" t="n">
         <f aca="false">D13*E13</f>
+        <v>0.5</v>
+      </c>
+      <c r="G13" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="J13" s="1"/>
+    </row>
+    <row r="14" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B14" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="C14" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D14" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" s="1" t="n">
         <v>6.13</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>16</v>
-      </c>
-    </row>
-    <row r="14" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B14" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="C14" s="4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E14" s="1" t="n">
-        <v>3.62</v>
       </c>
       <c r="F14" s="3" t="n">
         <f aca="false">D14*E14</f>
-        <v>3.62</v>
+        <v>6.13</v>
       </c>
       <c r="G14" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B15" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="C15" s="4" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="D15" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E15" s="1" t="n">
-        <v>2.39</v>
+        <v>3.62</v>
       </c>
       <c r="F15" s="3" t="n">
         <f aca="false">D15*E15</f>
+        <v>3.62</v>
+      </c>
+      <c r="G15" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B16" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="C16" s="4" t="s">
+        <v>25</v>
+      </c>
+      <c r="D16" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E16" s="1" t="n">
         <v>2.39</v>
-      </c>
-    </row>
-    <row r="16" customFormat="false" ht="45.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B16" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="C16" s="4" t="s">
-        <v>23</v>
-      </c>
-      <c r="D16" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E16" s="1" t="n">
-        <v>2.51</v>
       </c>
       <c r="F16" s="3" t="n">
         <f aca="false">D16*E16</f>
+        <v>2.39</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="46.25" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B17" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D17" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E17" s="1" t="n">
         <v>2.51</v>
-      </c>
-      <c r="G16" s="1" t="s">
-        <v>24</v>
-      </c>
-    </row>
-    <row r="17" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="B17" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="C17" s="4" t="s">
-        <v>26</v>
-      </c>
-      <c r="D17" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E17" s="1" t="n">
-        <v>0.6</v>
       </c>
       <c r="F17" s="3" t="n">
         <f aca="false">D17*E17</f>
-        <v>0.6</v>
+        <v>2.51</v>
       </c>
       <c r="G17" s="1" t="s">
-        <v>27</v>
-      </c>
-    </row>
-    <row r="18" customFormat="false" ht="28.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B18" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C18" s="4" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="D18" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E18" s="1" t="n">
-        <v>0.36</v>
+        <v>0.49</v>
       </c>
       <c r="F18" s="3" t="n">
         <f aca="false">D18*E18</f>
-        <v>0.36</v>
+        <v>0.49</v>
       </c>
       <c r="G18" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="19" customFormat="false" ht="23.3" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B19" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="C19" s="4" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D19" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E19" s="1" t="n">
-        <v>0.21</v>
+        <v>0.6</v>
       </c>
       <c r="F19" s="3" t="n">
         <f aca="false">D19*E19</f>
-        <v>0.21</v>
+        <v>0.6</v>
       </c>
       <c r="G19" s="1" t="s">
-        <v>33</v>
-      </c>
-    </row>
-    <row r="20" customFormat="false" ht="23.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>34</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="28.9" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B20" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C20" s="4" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="D20" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E20" s="1" t="n">
-        <v>0.51</v>
+        <v>0.36</v>
       </c>
       <c r="F20" s="3" t="n">
         <f aca="false">D20*E20</f>
-        <v>0.51</v>
+        <v>0.36</v>
       </c>
       <c r="G20" s="1" t="s">
-        <v>36</v>
-      </c>
-    </row>
-    <row r="21" customFormat="false" ht="23.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="21" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B21" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C21" s="4" t="s">
-        <v>38</v>
+        <v>39</v>
+      </c>
+      <c r="D21" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E21" s="1" t="n">
+        <v>0.21</v>
       </c>
       <c r="F21" s="3" t="n">
         <f aca="false">D21*E21</f>
-        <v>0</v>
+        <v>0.21</v>
       </c>
       <c r="G21" s="1" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="22" customFormat="false" ht="23.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="22" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="B22" s="1" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C22" s="4" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D22" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="1" t="n">
-        <v>3.54</v>
+        <v>0.51</v>
       </c>
       <c r="F22" s="3" t="n">
         <f aca="false">D22*E22</f>
-        <v>3.54</v>
+        <v>0.51</v>
       </c>
       <c r="G22" s="1" t="s">
-        <v>42</v>
-      </c>
-    </row>
-    <row r="23" customFormat="false" ht="23.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="23" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B23" s="1" t="s">
+        <v>44</v>
+      </c>
       <c r="C23" s="4" t="s">
-        <v>43</v>
-      </c>
-      <c r="D23" s="1" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="1" t="n">
-        <v>2.44</v>
+        <v>45</v>
       </c>
       <c r="F23" s="3" t="n">
         <f aca="false">D23*E23</f>
-        <v>2.44</v>
+        <v>0</v>
       </c>
       <c r="G23" s="1" t="s">
-        <v>44</v>
-      </c>
-    </row>
-    <row r="24" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C24" s="4"/>
+        <v>46</v>
+      </c>
+    </row>
+    <row r="24" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B24" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C24" s="4" t="s">
+        <v>48</v>
+      </c>
+      <c r="D24" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E24" s="1" t="n">
+        <v>3.54</v>
+      </c>
       <c r="F24" s="3" t="n">
         <f aca="false">D24*E24</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="25" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+        <v>3.54</v>
+      </c>
+      <c r="G24" s="1" t="s">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="25" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C25" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D25" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="1" t="n">
+        <v>2.44</v>
+      </c>
       <c r="F25" s="3" t="n">
         <f aca="false">D25*E25</f>
-        <v>0</v>
+        <v>2.44</v>
+      </c>
+      <c r="G25" s="1" t="s">
+        <v>51</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B26" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="C26" s="4" t="s">
+        <v>53</v>
+      </c>
+      <c r="D26" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E26" s="1" t="n">
+        <v>2.75</v>
+      </c>
       <c r="F26" s="3" t="n">
         <f aca="false">D26*E26</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C27" s="4"/>
+        <v>2.75</v>
+      </c>
+      <c r="G26" s="1" t="s">
+        <v>54</v>
+      </c>
+    </row>
+    <row r="27" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="B27" s="0" t="s">
+        <v>56</v>
+      </c>
+      <c r="C27" s="0" t="s">
+        <v>57</v>
+      </c>
+      <c r="D27" s="0" t="n">
+        <v>1</v>
+      </c>
+      <c r="E27" s="0" t="n">
+        <v>1.09</v>
+      </c>
       <c r="F27" s="3" t="n">
         <f aca="false">D27*E27</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="28" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C28" s="4"/>
+        <v>1.09</v>
+      </c>
+      <c r="G27" s="0" t="s">
+        <v>58</v>
+      </c>
+    </row>
+    <row r="28" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="1"/>
+      <c r="B28" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="C28" s="4" t="s">
+        <v>60</v>
+      </c>
+      <c r="D28" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E28" s="1" t="n">
+        <v>0.33</v>
+      </c>
       <c r="F28" s="3" t="n">
         <f aca="false">D28*E28</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="29" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C29" s="4"/>
+        <v>0.33</v>
+      </c>
+      <c r="G28" s="1" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="29" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B29" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C29" s="4" t="s">
+        <v>63</v>
+      </c>
+      <c r="D29" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E29" s="1" t="n">
+        <v>0.33</v>
+      </c>
       <c r="F29" s="3" t="n">
         <f aca="false">D29*E29</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="30" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C30" s="5"/>
-    </row>
-    <row r="31" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C31" s="5"/>
+        <v>0.66</v>
+      </c>
+      <c r="G29" s="1" t="s">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="30" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B30" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C30" s="4" t="s">
+        <v>66</v>
+      </c>
+      <c r="D30" s="1" t="n">
+        <v>5</v>
+      </c>
+      <c r="E30" s="1" t="n">
+        <v>0.11</v>
+      </c>
+      <c r="F30" s="3" t="n">
+        <f aca="false">D30*E30</f>
+        <v>0.55</v>
+      </c>
+      <c r="G30" s="1" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="31" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="B31" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C31" s="4" t="s">
+        <v>69</v>
+      </c>
+      <c r="D31" s="1" t="n">
+        <v>6</v>
+      </c>
+      <c r="E31" s="1" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F31" s="3" t="n">
+        <f aca="false">D31*E31</f>
+        <v>0.78</v>
+      </c>
+      <c r="G31" s="1" t="s">
+        <v>70</v>
+      </c>
     </row>
     <row r="32" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="B32" s="2" t="s">
-        <v>4</v>
-      </c>
-      <c r="C32" s="6"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2" t="n">
-        <f aca="false">SUM(F11:F31)</f>
-        <v>23.31</v>
-      </c>
-      <c r="G32" s="7"/>
-    </row>
-    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C33" s="5"/>
+      <c r="B32" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C32" s="3" t="s">
+        <v>72</v>
+      </c>
+      <c r="D32" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="E32" s="1" t="n">
+        <v>0.08</v>
+      </c>
+      <c r="F32" s="3" t="n">
+        <f aca="false">D32*E32</f>
+        <v>0.56</v>
+      </c>
+      <c r="G32" s="1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="33" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B33" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="C33" s="3" t="s">
+        <v>75</v>
+      </c>
+      <c r="D33" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E33" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F33" s="3" t="n">
+        <f aca="false">D33*E33</f>
+        <v>0.1</v>
+      </c>
+      <c r="G33" s="1" t="s">
+        <v>76</v>
+      </c>
     </row>
     <row r="34" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C34" s="5"/>
+      <c r="B34" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>78</v>
+      </c>
+      <c r="D34" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E34" s="1" t="n">
+        <v>0.13</v>
+      </c>
+      <c r="F34" s="3" t="n">
+        <f aca="false">D34*E34</f>
+        <v>0.13</v>
+      </c>
+      <c r="G34" s="1" t="s">
+        <v>79</v>
+      </c>
     </row>
     <row r="35" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C35" s="5"/>
+      <c r="B35" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>81</v>
+      </c>
+      <c r="D35" s="1" t="n">
+        <v>7</v>
+      </c>
+      <c r="E35" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F35" s="3" t="n">
+        <f aca="false">D35*E35</f>
+        <v>0.7</v>
+      </c>
+      <c r="G35" s="1" t="s">
+        <v>82</v>
+      </c>
     </row>
     <row r="36" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C36" s="5"/>
+      <c r="B36" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>84</v>
+      </c>
+      <c r="D36" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E36" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F36" s="3" t="n">
+        <f aca="false">D36*E36</f>
+        <v>0.2</v>
+      </c>
+      <c r="G36" s="1" t="s">
+        <v>85</v>
+      </c>
     </row>
     <row r="37" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C37" s="4"/>
+      <c r="B37" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C37" s="3" t="s">
+        <v>87</v>
+      </c>
+      <c r="D37" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E37" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F37" s="3" t="n">
+        <f aca="false">D37*E37</f>
+        <v>0.1</v>
+      </c>
+      <c r="G37" s="1" t="s">
+        <v>88</v>
+      </c>
     </row>
     <row r="38" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C38" s="4"/>
+      <c r="B38" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C38" s="3" t="s">
+        <v>90</v>
+      </c>
+      <c r="D38" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E38" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F38" s="3" t="n">
+        <f aca="false">D38*E38</f>
+        <v>0.1</v>
+      </c>
+      <c r="G38" s="1" t="s">
+        <v>91</v>
+      </c>
     </row>
     <row r="39" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B39" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C39" s="4"/>
+        <v>92</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>93</v>
+      </c>
+      <c r="D39" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E39" s="1" t="n">
+        <v>0.1</v>
+      </c>
       <c r="F39" s="3" t="n">
         <f aca="false">D39*E39</f>
-        <v>0</v>
+        <v>0.4</v>
+      </c>
+      <c r="G39" s="1" t="s">
+        <v>94</v>
       </c>
     </row>
     <row r="40" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B40" s="1" t="s">
-        <v>46</v>
-      </c>
-      <c r="C40" s="4"/>
+        <v>95</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>96</v>
+      </c>
+      <c r="D40" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E40" s="1" t="n">
+        <v>0.1</v>
+      </c>
       <c r="F40" s="3" t="n">
         <f aca="false">D40*E40</f>
-        <v>0</v>
-      </c>
-      <c r="G40" s="8" t="s">
-        <v>47</v>
+        <v>0.2</v>
+      </c>
+      <c r="G40" s="1" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="41" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B41" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C41" s="4" t="s">
-        <v>49</v>
+        <v>98</v>
+      </c>
+      <c r="C41" s="3" t="s">
+        <v>99</v>
       </c>
       <c r="D41" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E41" s="1" t="n">
-        <v>1.9</v>
+        <v>0.1</v>
       </c>
       <c r="F41" s="3" t="n">
         <f aca="false">D41*E41</f>
-        <v>1.9</v>
+        <v>0.1</v>
       </c>
       <c r="G41" s="1" t="s">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="42" customFormat="false" ht="23.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="C42" s="4" t="s">
-        <v>43</v>
+        <v>100</v>
+      </c>
+    </row>
+    <row r="42" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B42" s="1" t="s">
+        <v>101</v>
+      </c>
+      <c r="C42" s="3" t="s">
+        <v>102</v>
       </c>
       <c r="D42" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E42" s="1" t="n">
-        <v>2.44</v>
+        <v>0.1</v>
       </c>
       <c r="F42" s="3" t="n">
         <f aca="false">D42*E42</f>
-        <v>2.44</v>
+        <v>0.1</v>
       </c>
       <c r="G42" s="1" t="s">
-        <v>44</v>
+        <v>103</v>
       </c>
     </row>
     <row r="43" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C43" s="4" t="s">
-        <v>51</v>
+      <c r="B43" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C43" s="3" t="s">
+        <v>105</v>
+      </c>
+      <c r="D43" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E43" s="1" t="n">
+        <v>0.1</v>
       </c>
       <c r="F43" s="3" t="n">
         <f aca="false">D43*E43</f>
-        <v>0</v>
+        <v>0.1</v>
+      </c>
+      <c r="G43" s="1" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="44" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
-      <c r="C44" s="4" t="s">
-        <v>52</v>
+      <c r="B44" s="1" t="s">
+        <v>107</v>
+      </c>
+      <c r="C44" s="3" t="s">
+        <v>108</v>
+      </c>
+      <c r="D44" s="1" t="n">
+        <v>2</v>
+      </c>
+      <c r="E44" s="1" t="n">
+        <v>0.1</v>
       </c>
       <c r="F44" s="3" t="n">
         <f aca="false">D44*E44</f>
-        <v>0</v>
+        <v>0.2</v>
+      </c>
+      <c r="G44" s="1" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="45" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="B45" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C45" s="4" t="s">
-        <v>54</v>
+        <v>110</v>
+      </c>
+      <c r="C45" s="3" t="s">
+        <v>111</v>
       </c>
       <c r="D45" s="1" t="n">
         <v>1</v>
       </c>
       <c r="E45" s="1" t="n">
-        <v>1.26</v>
+        <v>0.1</v>
       </c>
       <c r="F45" s="3" t="n">
         <f aca="false">D45*E45</f>
+        <v>0.1</v>
+      </c>
+      <c r="G45" s="1" t="s">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="46" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B46" s="1" t="s">
+        <v>113</v>
+      </c>
+      <c r="C46" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D46" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E46" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F46" s="3" t="n">
+        <f aca="false">D46*E46</f>
+        <v>0.1</v>
+      </c>
+      <c r="G46" s="1" t="s">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="47" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B47" s="1" t="s">
+        <v>116</v>
+      </c>
+      <c r="C47" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D47" s="1" t="n">
+        <v>9</v>
+      </c>
+      <c r="E47" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F47" s="3" t="n">
+        <f aca="false">D47*E47</f>
+        <v>0.9</v>
+      </c>
+      <c r="G47" s="1" t="s">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="48" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B48" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C48" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D48" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E48" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F48" s="3" t="n">
+        <f aca="false">D48*E48</f>
+        <v>0.3</v>
+      </c>
+      <c r="G48" s="1" t="s">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="49" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B49" s="1" t="s">
+        <v>122</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D49" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E49" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F49" s="3" t="n">
+        <f aca="false">D49*E49</f>
+        <v>0.1</v>
+      </c>
+      <c r="G49" s="1" t="s">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="50" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B50" s="1" t="s">
+        <v>125</v>
+      </c>
+      <c r="C50" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D50" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E50" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F50" s="3" t="n">
+        <f aca="false">D50*E50</f>
+        <v>0.1</v>
+      </c>
+      <c r="G50" s="1" t="s">
+        <v>127</v>
+      </c>
+    </row>
+    <row r="51" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B51" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="C51" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D51" s="1" t="n">
+        <v>4</v>
+      </c>
+      <c r="E51" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F51" s="3" t="n">
+        <f aca="false">D51*E51</f>
+        <v>0.4</v>
+      </c>
+      <c r="G51" s="1" t="s">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="52" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B52" s="1" t="s">
+        <v>131</v>
+      </c>
+      <c r="C52" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D52" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E52" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F52" s="3" t="n">
+        <f aca="false">D52*E52</f>
+        <v>0.1</v>
+      </c>
+      <c r="G52" s="1" t="s">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="53" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B53" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="C53" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D53" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E53" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F53" s="3" t="n">
+        <f aca="false">D53*E53</f>
+        <v>0.3</v>
+      </c>
+      <c r="G53" s="1" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="54" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B54" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D54" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E54" s="1" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F54" s="3" t="n">
+        <f aca="false">D54*E54</f>
+        <v>0.3</v>
+      </c>
+      <c r="G54" s="1" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="55" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B55" s="5" t="n">
+        <v>1935161</v>
+      </c>
+      <c r="C55" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D55" s="1" t="n">
+        <v>3</v>
+      </c>
+      <c r="E55" s="1" t="n">
+        <v>0.53</v>
+      </c>
+      <c r="F55" s="3" t="n">
+        <f aca="false">D55*E55</f>
+        <v>1.59</v>
+      </c>
+      <c r="G55" s="1" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="56" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C56" s="3"/>
+      <c r="F56" s="3" t="n">
+        <f aca="false">D56*E56</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="59" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B59" s="2" t="s">
+        <v>4</v>
+      </c>
+      <c r="C59" s="6"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2" t="n">
+        <f aca="false">SUM(F11:F58)</f>
+        <v>41.78</v>
+      </c>
+      <c r="G59" s="7"/>
+    </row>
+    <row r="60" customFormat="false" ht="12.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C60" s="4"/>
+    </row>
+    <row r="61" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C61" s="4"/>
+    </row>
+    <row r="62" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C62" s="4"/>
+    </row>
+    <row r="63" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C63" s="4"/>
+    </row>
+    <row r="64" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C64" s="4"/>
+    </row>
+    <row r="65" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C65" s="4"/>
+    </row>
+    <row r="66" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B66" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="C66" s="4"/>
+      <c r="F66" s="3" t="n">
+        <f aca="false">D66*E66</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="67" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B67" s="1" t="s">
+        <v>143</v>
+      </c>
+      <c r="C67" s="4"/>
+      <c r="F67" s="3" t="n">
+        <f aca="false">D67*E67</f>
+        <v>0</v>
+      </c>
+      <c r="G67" s="8" t="s">
+        <v>144</v>
+      </c>
+    </row>
+    <row r="68" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B68" s="1" t="s">
+        <v>145</v>
+      </c>
+      <c r="C68" s="4" t="s">
+        <v>146</v>
+      </c>
+      <c r="D68" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E68" s="1" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F68" s="3" t="n">
+        <f aca="false">D68*E68</f>
+        <v>1.9</v>
+      </c>
+      <c r="G68" s="1" t="s">
+        <v>147</v>
+      </c>
+    </row>
+    <row r="69" customFormat="false" ht="23.45" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="C69" s="4" t="s">
+        <v>50</v>
+      </c>
+      <c r="D69" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E69" s="1" t="n">
+        <v>2.44</v>
+      </c>
+      <c r="F69" s="3" t="n">
+        <f aca="false">D69*E69</f>
+        <v>2.44</v>
+      </c>
+      <c r="G69" s="1" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="70" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C70" s="4" t="s">
+        <v>148</v>
+      </c>
+      <c r="F70" s="3" t="n">
+        <f aca="false">D70*E70</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="71" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="C71" s="4" t="s">
+        <v>149</v>
+      </c>
+      <c r="F71" s="3" t="n">
+        <f aca="false">D71*E71</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="72" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B72" s="1" t="s">
+        <v>150</v>
+      </c>
+      <c r="C72" s="4" t="s">
+        <v>151</v>
+      </c>
+      <c r="D72" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E72" s="1" t="n">
         <v>1.26</v>
       </c>
-      <c r="G45" s="9" t="s">
-        <v>55</v>
+      <c r="F72" s="3" t="n">
+        <f aca="false">D72*E72</f>
+        <v>1.26</v>
+      </c>
+      <c r="G72" s="9" t="s">
+        <v>152</v>
+      </c>
+    </row>
+    <row r="75" customFormat="false" ht="12.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="B75" s="1" t="s">
+        <v>153</v>
+      </c>
+      <c r="C75" s="4" t="s">
+        <v>154</v>
+      </c>
+      <c r="D75" s="1" t="n">
+        <v>1</v>
+      </c>
+      <c r="E75" s="1" t="n">
+        <v>1.36</v>
+      </c>
+      <c r="F75" s="3" t="n">
+        <f aca="false">D75*E75</f>
+        <v>1.36</v>
+      </c>
+      <c r="G75" s="1" t="s">
+        <v>155</v>
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A10:G56"/>
   <hyperlinks>
-    <hyperlink ref="G45" r:id="rId1" display="https://www.digikey.com/short/fd05pjh9"/>
+    <hyperlink ref="G72" r:id="rId1" display="https://www.digikey.com/short/fd05pjh9"/>
   </hyperlinks>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.7875" right="0.7875" top="1.05277777777778" bottom="1.05277777777778" header="0.7875" footer="0.7875"/>
@@ -1290,6 +2275,7 @@
     <oddHeader>&amp;C&amp;"Times New Roman,Regular"&amp;12&amp;A</oddHeader>
     <oddFooter>&amp;C&amp;"Times New Roman,Regular"&amp;12Page &amp;P</oddFooter>
   </headerFooter>
+  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -1303,7 +2289,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="10" t="s">
-        <v>56</v>
+        <v>156</v>
       </c>
       <c r="B1" s="10"/>
       <c r="C1" s="10"/>
@@ -1316,7 +2302,7 @@
     </row>
     <row r="2" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A2" s="11" t="s">
-        <v>57</v>
+        <v>157</v>
       </c>
       <c r="B2" s="11"/>
       <c r="C2" s="11"/>
@@ -1329,12 +2315,12 @@
     </row>
     <row r="4" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="12" t="s">
-        <v>58</v>
+        <v>158</v>
       </c>
       <c r="B4" s="13"/>
       <c r="C4" s="13"/>
       <c r="D4" s="12" t="s">
-        <v>59</v>
+        <v>159</v>
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="13"/>
@@ -1345,14 +2331,14 @@
     </row>
     <row r="5" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="14" t="s">
-        <v>60</v>
+        <v>160</v>
       </c>
       <c r="B5" s="15" t="n">
         <v>459</v>
       </c>
       <c r="C5" s="13"/>
       <c r="D5" s="14" t="s">
-        <v>61</v>
+        <v>161</v>
       </c>
       <c r="E5" s="16" t="n">
         <f aca="false">1/(1/($B$6/($B$15/1000))-1/$B$10)</f>
@@ -1366,14 +2352,14 @@
     </row>
     <row r="6" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="14" t="s">
-        <v>62</v>
+        <v>162</v>
       </c>
       <c r="B6" s="15" t="n">
         <v>478</v>
       </c>
       <c r="C6" s="13"/>
       <c r="D6" s="14" t="s">
-        <v>63</v>
+        <v>163</v>
       </c>
       <c r="E6" s="16" t="n">
         <f aca="false">1/(1/($B$6/($B$16/1000))-1/$B$10-1/$E$5)</f>
@@ -1387,7 +2373,7 @@
     </row>
     <row r="7" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="14" t="s">
-        <v>64</v>
+        <v>164</v>
       </c>
       <c r="B7" s="15" t="n">
         <v>500</v>
@@ -1403,14 +2389,14 @@
     </row>
     <row r="8" customFormat="false" ht="35.05" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="14" t="s">
-        <v>65</v>
+        <v>165</v>
       </c>
       <c r="B8" s="17" t="n">
         <v>0.01</v>
       </c>
       <c r="C8" s="13"/>
       <c r="D8" s="14" t="s">
-        <v>66</v>
+        <v>166</v>
       </c>
       <c r="E8" s="18" t="n">
         <f aca="false">($B$11/$E$5)-1</f>
@@ -1427,7 +2413,7 @@
       <c r="B9" s="13"/>
       <c r="C9" s="13"/>
       <c r="D9" s="14" t="s">
-        <v>67</v>
+        <v>167</v>
       </c>
       <c r="E9" s="18" t="n">
         <f aca="false">($B$12/$E$6)-1</f>
@@ -1441,7 +2427,7 @@
     </row>
     <row r="10" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="14" t="s">
-        <v>68</v>
+        <v>168</v>
       </c>
       <c r="B10" s="15" t="n">
         <v>1050</v>
@@ -1457,7 +2443,7 @@
     </row>
     <row r="11" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="14" t="s">
-        <v>69</v>
+        <v>169</v>
       </c>
       <c r="B11" s="15" t="n">
         <v>201</v>
@@ -1473,7 +2459,7 @@
     </row>
     <row r="12" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="14" t="s">
-        <v>70</v>
+        <v>170</v>
       </c>
       <c r="B12" s="15" t="n">
         <v>504</v>
@@ -1501,7 +2487,7 @@
     </row>
     <row r="14" customFormat="false" ht="34.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="14" t="s">
-        <v>71</v>
+        <v>171</v>
       </c>
       <c r="B14" s="15" t="n">
         <v>500</v>
@@ -1517,7 +2503,7 @@
     </row>
     <row r="15" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="14" t="s">
-        <v>72</v>
+        <v>172</v>
       </c>
       <c r="B15" s="15" t="n">
         <v>1500</v>
@@ -1533,7 +2519,7 @@
     </row>
     <row r="16" customFormat="false" ht="23.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="14" t="s">
-        <v>73</v>
+        <v>173</v>
       </c>
       <c r="B16" s="15" t="n">
         <v>3000</v>
@@ -1585,45 +2571,45 @@
     </row>
     <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="19" t="s">
-        <v>74</v>
+        <v>174</v>
       </c>
       <c r="B20" s="19" t="s">
-        <v>75</v>
+        <v>175</v>
       </c>
       <c r="C20" s="19" t="s">
-        <v>76</v>
+        <v>176</v>
       </c>
       <c r="D20" s="19" t="s">
-        <v>77</v>
+        <v>177</v>
       </c>
       <c r="E20" s="19" t="s">
-        <v>78</v>
+        <v>178</v>
       </c>
       <c r="F20" s="19" t="s">
-        <v>79</v>
+        <v>179</v>
       </c>
       <c r="G20" s="19" t="s">
-        <v>80</v>
+        <v>180</v>
       </c>
       <c r="H20" s="19" t="s">
-        <v>81</v>
+        <v>181</v>
       </c>
       <c r="I20" s="19" t="s">
-        <v>82</v>
+        <v>182</v>
       </c>
       <c r="J20" s="19" t="s">
-        <v>83</v>
+        <v>183</v>
       </c>
     </row>
     <row r="21" customFormat="false" ht="45.75" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="20" t="s">
-        <v>84</v>
+        <v>184</v>
       </c>
       <c r="B21" s="21" t="s">
-        <v>85</v>
+        <v>185</v>
       </c>
       <c r="C21" s="21" t="s">
-        <v>86</v>
+        <v>186</v>
       </c>
       <c r="D21" s="22" t="n">
         <f aca="false">$B$10</f>
@@ -1656,13 +2642,13 @@
     </row>
     <row r="22" customFormat="false" ht="13.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="20" t="s">
-        <v>87</v>
+        <v>187</v>
       </c>
       <c r="B22" s="21" t="s">
-        <v>88</v>
+        <v>188</v>
       </c>
       <c r="C22" s="21" t="s">
-        <v>85</v>
+        <v>185</v>
       </c>
       <c r="D22" s="22" t="n">
         <f aca="false">1/(1/$B$10+1/$B$11)</f>
@@ -1695,13 +2681,13 @@
     </row>
     <row r="23" customFormat="false" ht="13.9" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="20" t="s">
-        <v>89</v>
+        <v>189</v>
       </c>
       <c r="B23" s="21" t="s">
-        <v>88</v>
+        <v>188</v>
       </c>
       <c r="C23" s="21" t="s">
-        <v>88</v>
+        <v>188</v>
       </c>
       <c r="D23" s="22" t="n">
         <f aca="false">1/(1/$B$10+1/$B$11+1/$B$12)</f>
@@ -1734,7 +2720,7 @@
     </row>
     <row r="26" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="24" t="s">
-        <v>90</v>
+        <v>190</v>
       </c>
       <c r="B26" s="25"/>
       <c r="C26" s="25"/>
@@ -1748,7 +2734,7 @@
     </row>
     <row r="27" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A27" s="26" t="s">
-        <v>91</v>
+        <v>191</v>
       </c>
       <c r="B27" s="26"/>
       <c r="C27" s="26"/>
@@ -1762,7 +2748,7 @@
     </row>
     <row r="28" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="26" t="s">
-        <v>92</v>
+        <v>192</v>
       </c>
       <c r="B28" s="26"/>
       <c r="C28" s="26"/>
@@ -1776,7 +2762,7 @@
     </row>
     <row r="29" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A29" s="26" t="s">
-        <v>93</v>
+        <v>193</v>
       </c>
       <c r="B29" s="26"/>
       <c r="C29" s="26"/>
@@ -1790,7 +2776,7 @@
     </row>
     <row r="30" customFormat="false" ht="13.8" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A30" s="26" t="s">
-        <v>94</v>
+        <v>194</v>
       </c>
       <c r="B30" s="26"/>
       <c r="C30" s="26"/>
@@ -1812,10 +2798,10 @@
     <mergeCell ref="A30:J30"/>
   </mergeCells>
   <conditionalFormatting sqref="J21:J23">
-    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="0">
+    <cfRule type="expression" priority="2" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="2">
       <formula>J21="OK"</formula>
     </cfRule>
-    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="1">
+    <cfRule type="expression" priority="3" aboveAverage="0" equalAverage="0" bottom="0" percent="0" rank="0" text="" dxfId="3">
       <formula>J21="CHECK"</formula>
     </cfRule>
   </conditionalFormatting>

</xml_diff>